<commit_message>
kalimai mandir valuation given
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/नगर बजेट estimate/कालिकामाई मन्दिर पूर्वाधार विकास/V-कालिकामाई मन्दिर पूर्वाधार विकास.xlsx
+++ b/बजेट माग estimate/नगर बजेट estimate/कालिकामाई मन्दिर पूर्वाधार विकास/V-कालिकामाई मन्दिर पूर्वाधार विकास.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43CC4712-67BF-4A7E-9DBB-2CE76AADCD06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{560C8237-DCF2-4535-974C-C50E8C6E57C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="estimate" sheetId="12" r:id="rId1"/>
@@ -367,10 +367,10 @@
     <t>Detail Quantity Measurement Sheet</t>
   </si>
   <si>
-    <t xml:space="preserve">Date:2083/03/15       </t>
+    <t xml:space="preserve">Date:2083/03/24       </t>
   </si>
   <si>
-    <t>Date: 2083/03/15</t>
+    <t>Date: 2083/03/24</t>
   </si>
 </sst>
 </file>
@@ -777,63 +777,8 @@
     <xf numFmtId="0" fontId="23" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -853,8 +798,63 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1618,113 +1618,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="74" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
+      <c r="F1" s="74"/>
+      <c r="G1" s="74"/>
+      <c r="H1" s="74"/>
+      <c r="I1" s="74"/>
+      <c r="J1" s="74"/>
+      <c r="K1" s="74"/>
     </row>
     <row r="2" spans="1:16" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="79" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
-      <c r="J2" s="79"/>
-      <c r="K2" s="79"/>
+      <c r="A2" s="75" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="75"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="75"/>
+      <c r="F2" s="75"/>
+      <c r="G2" s="75"/>
+      <c r="H2" s="75"/>
+      <c r="I2" s="75"/>
+      <c r="J2" s="75"/>
+      <c r="K2" s="75"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="80" t="s">
+      <c r="A3" s="76" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="80"/>
-      <c r="C3" s="80"/>
-      <c r="D3" s="80"/>
-      <c r="E3" s="80"/>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
-      <c r="H3" s="80"/>
-      <c r="I3" s="80"/>
-      <c r="J3" s="80"/>
-      <c r="K3" s="80"/>
+      <c r="B3" s="76"/>
+      <c r="C3" s="76"/>
+      <c r="D3" s="76"/>
+      <c r="E3" s="76"/>
+      <c r="F3" s="76"/>
+      <c r="G3" s="76"/>
+      <c r="H3" s="76"/>
+      <c r="I3" s="76"/>
+      <c r="J3" s="76"/>
+      <c r="K3" s="76"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="80" t="s">
+      <c r="A4" s="76" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="80"/>
-      <c r="C4" s="80"/>
-      <c r="D4" s="80"/>
-      <c r="E4" s="80"/>
-      <c r="F4" s="80"/>
-      <c r="G4" s="80"/>
-      <c r="H4" s="80"/>
-      <c r="I4" s="80"/>
-      <c r="J4" s="80"/>
-      <c r="K4" s="80"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="76"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="76"/>
+      <c r="F4" s="76"/>
+      <c r="G4" s="76"/>
+      <c r="H4" s="76"/>
+      <c r="I4" s="76"/>
+      <c r="J4" s="76"/>
+      <c r="K4" s="76"/>
     </row>
     <row r="5" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="81" t="s">
+      <c r="A5" s="77" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="81"/>
-      <c r="C5" s="81"/>
-      <c r="D5" s="81"/>
-      <c r="E5" s="81"/>
-      <c r="F5" s="81"/>
-      <c r="G5" s="81"/>
-      <c r="H5" s="81"/>
-      <c r="I5" s="81"/>
-      <c r="J5" s="81"/>
-      <c r="K5" s="81"/>
+      <c r="B5" s="77"/>
+      <c r="C5" s="77"/>
+      <c r="D5" s="77"/>
+      <c r="E5" s="77"/>
+      <c r="F5" s="77"/>
+      <c r="G5" s="77"/>
+      <c r="H5" s="77"/>
+      <c r="I5" s="77"/>
+      <c r="J5" s="77"/>
+      <c r="K5" s="77"/>
     </row>
     <row r="6" spans="1:16" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="68" t="s">
+      <c r="A6" s="72" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="68"/>
-      <c r="C6" s="68"/>
-      <c r="D6" s="68"/>
-      <c r="E6" s="68"/>
-      <c r="F6" s="68"/>
+      <c r="B6" s="72"/>
+      <c r="C6" s="72"/>
+      <c r="D6" s="72"/>
+      <c r="E6" s="72"/>
+      <c r="F6" s="72"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="77" t="s">
+      <c r="H6" s="73" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="77"/>
-      <c r="J6" s="77"/>
-      <c r="K6" s="77"/>
+      <c r="I6" s="73"/>
+      <c r="J6" s="73"/>
+      <c r="K6" s="73"/>
     </row>
     <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="84" t="s">
+      <c r="A7" s="67" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="84"/>
-      <c r="C7" s="84"/>
-      <c r="D7" s="84"/>
-      <c r="E7" s="84"/>
-      <c r="F7" s="84"/>
+      <c r="B7" s="67"/>
+      <c r="C7" s="67"/>
+      <c r="D7" s="67"/>
+      <c r="E7" s="67"/>
+      <c r="F7" s="67"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="85" t="s">
+      <c r="H7" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="I7" s="85"/>
-      <c r="J7" s="85"/>
-      <c r="K7" s="85"/>
+      <c r="I7" s="68"/>
+      <c r="J7" s="68"/>
+      <c r="K7" s="68"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
@@ -3483,11 +3483,11 @@
       <c r="B83" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="C83" s="82">
+      <c r="C83" s="65">
         <f>J81</f>
         <v>569007.79144636379</v>
       </c>
-      <c r="D83" s="83"/>
+      <c r="D83" s="66"/>
       <c r="E83" s="9">
         <v>100</v>
       </c>
@@ -3509,21 +3509,21 @@
       <c r="B84" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C84" s="86">
+      <c r="C84" s="69">
         <v>500000</v>
       </c>
-      <c r="D84" s="87"/>
+      <c r="D84" s="70"/>
       <c r="E84" s="9"/>
     </row>
     <row r="85" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B85" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C85" s="86">
+      <c r="C85" s="69">
         <f>C84-C87-C88</f>
         <v>475000</v>
       </c>
-      <c r="D85" s="87"/>
+      <c r="D85" s="70"/>
       <c r="E85" s="9">
         <f>C85/C83*100</f>
         <v>83.47864601161173</v>
@@ -3533,11 +3533,11 @@
       <c r="B86" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="C86" s="88">
+      <c r="C86" s="71">
         <f>C83-C85</f>
         <v>94007.791446363786</v>
       </c>
-      <c r="D86" s="88"/>
+      <c r="D86" s="71"/>
       <c r="E86" s="9">
         <f>100-E85</f>
         <v>16.52135398838827</v>
@@ -3547,11 +3547,11 @@
       <c r="B87" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C87" s="82">
+      <c r="C87" s="65">
         <f>C84*0.03</f>
         <v>15000</v>
       </c>
-      <c r="D87" s="83"/>
+      <c r="D87" s="66"/>
       <c r="E87" s="9">
         <v>3</v>
       </c>
@@ -3560,17 +3560,24 @@
       <c r="B88" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C88" s="82">
+      <c r="C88" s="65">
         <f>C84*0.02</f>
         <v>10000</v>
       </c>
-      <c r="D88" s="83"/>
+      <c r="D88" s="66"/>
       <c r="E88" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C87:D87"/>
     <mergeCell ref="C88:D88"/>
     <mergeCell ref="A7:F7"/>
@@ -3579,13 +3586,6 @@
     <mergeCell ref="C84:D84"/>
     <mergeCell ref="C85:D85"/>
     <mergeCell ref="C86:D86"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
@@ -3615,90 +3615,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="71" t="s">
+      <c r="A1" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="71"/>
-      <c r="K1" s="71"/>
+      <c r="B1" s="80"/>
+      <c r="C1" s="80"/>
+      <c r="D1" s="80"/>
+      <c r="E1" s="80"/>
+      <c r="F1" s="80"/>
+      <c r="G1" s="80"/>
+      <c r="H1" s="80"/>
+      <c r="I1" s="80"/>
+      <c r="J1" s="80"/>
+      <c r="K1" s="80"/>
     </row>
     <row r="2" spans="1:13" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="72" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="72"/>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="72"/>
+      <c r="A2" s="81" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="81"/>
+      <c r="C2" s="81"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="81"/>
+      <c r="G2" s="81"/>
+      <c r="H2" s="81"/>
+      <c r="I2" s="81"/>
+      <c r="J2" s="81"/>
+      <c r="K2" s="81"/>
     </row>
     <row r="3" spans="1:13" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="73" t="s">
+      <c r="A3" s="82" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="73"/>
-      <c r="C3" s="73"/>
-      <c r="D3" s="73"/>
-      <c r="E3" s="73"/>
-      <c r="F3" s="73"/>
-      <c r="G3" s="73"/>
-      <c r="H3" s="73"/>
-      <c r="I3" s="73"/>
-      <c r="J3" s="73"/>
-      <c r="K3" s="73"/>
+      <c r="B3" s="82"/>
+      <c r="C3" s="82"/>
+      <c r="D3" s="82"/>
+      <c r="E3" s="82"/>
+      <c r="F3" s="82"/>
+      <c r="G3" s="82"/>
+      <c r="H3" s="82"/>
+      <c r="I3" s="82"/>
+      <c r="J3" s="82"/>
+      <c r="K3" s="82"/>
     </row>
     <row r="4" spans="1:13" s="43" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="73" t="s">
+      <c r="A4" s="82" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="73"/>
-      <c r="C4" s="73"/>
-      <c r="D4" s="73"/>
-      <c r="E4" s="73"/>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73"/>
-      <c r="H4" s="73"/>
-      <c r="I4" s="73"/>
-      <c r="J4" s="73"/>
-      <c r="K4" s="73"/>
+      <c r="B4" s="82"/>
+      <c r="C4" s="82"/>
+      <c r="D4" s="82"/>
+      <c r="E4" s="82"/>
+      <c r="F4" s="82"/>
+      <c r="G4" s="82"/>
+      <c r="H4" s="82"/>
+      <c r="I4" s="82"/>
+      <c r="J4" s="82"/>
+      <c r="K4" s="82"/>
     </row>
     <row r="5" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="74" t="s">
+      <c r="A5" s="83" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="74"/>
-      <c r="C5" s="74"/>
-      <c r="D5" s="74"/>
-      <c r="E5" s="74"/>
-      <c r="F5" s="74"/>
-      <c r="G5" s="74"/>
-      <c r="H5" s="74"/>
-      <c r="I5" s="74"/>
-      <c r="J5" s="74"/>
-      <c r="K5" s="74"/>
+      <c r="B5" s="83"/>
+      <c r="C5" s="83"/>
+      <c r="D5" s="83"/>
+      <c r="E5" s="83"/>
+      <c r="F5" s="83"/>
+      <c r="G5" s="83"/>
+      <c r="H5" s="83"/>
+      <c r="I5" s="83"/>
+      <c r="J5" s="83"/>
+      <c r="K5" s="83"/>
     </row>
     <row r="6" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="44" t="s">
         <v>70</v>
       </c>
       <c r="B6" s="44"/>
-      <c r="C6" s="75">
+      <c r="C6" s="78">
         <f>F55</f>
         <v>569007.79144636379</v>
       </c>
-      <c r="D6" s="76"/>
+      <c r="D6" s="79"/>
       <c r="E6" s="45"/>
       <c r="F6" s="44"/>
       <c r="G6" s="44"/>
@@ -3706,11 +3706,11 @@
         <v>71</v>
       </c>
       <c r="I6" s="44"/>
-      <c r="J6" s="75">
+      <c r="J6" s="78">
         <f>I55</f>
         <v>569089.07039927552</v>
       </c>
-      <c r="K6" s="76"/>
+      <c r="K6" s="79"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="46" t="s">
@@ -3719,76 +3719,76 @@
       <c r="B7" s="46"/>
       <c r="C7" s="46"/>
       <c r="D7" s="46"/>
-      <c r="F7" s="66"/>
-      <c r="G7" s="66"/>
-      <c r="I7" s="67" t="s">
+      <c r="F7" s="84"/>
+      <c r="G7" s="84"/>
+      <c r="I7" s="85" t="s">
         <v>73</v>
       </c>
-      <c r="J7" s="67"/>
-      <c r="K7" s="67"/>
+      <c r="J7" s="85"/>
+      <c r="K7" s="85"/>
     </row>
     <row r="8" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="68" t="s">
+      <c r="A8" s="72" t="s">
         <v>82</v>
       </c>
-      <c r="B8" s="68"/>
-      <c r="C8" s="68"/>
-      <c r="D8" s="68"/>
-      <c r="E8" s="68"/>
-      <c r="F8" s="68"/>
-      <c r="I8" s="69" t="s">
+      <c r="B8" s="72"/>
+      <c r="C8" s="72"/>
+      <c r="D8" s="72"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="72"/>
+      <c r="I8" s="86" t="s">
         <v>74</v>
       </c>
-      <c r="J8" s="69"/>
-      <c r="K8" s="69"/>
+      <c r="J8" s="86"/>
+      <c r="K8" s="86"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="70" t="str">
+      <c r="A9" s="87" t="str">
         <f>[7]estimate!A7</f>
         <v>Location:- Shankharapur Municipality 1</v>
       </c>
-      <c r="B9" s="70"/>
-      <c r="C9" s="70"/>
-      <c r="D9" s="70"/>
-      <c r="E9" s="70"/>
-      <c r="F9" s="70"/>
-      <c r="I9" s="69" t="s">
+      <c r="B9" s="87"/>
+      <c r="C9" s="87"/>
+      <c r="D9" s="87"/>
+      <c r="E9" s="87"/>
+      <c r="F9" s="87"/>
+      <c r="I9" s="86" t="s">
         <v>87</v>
       </c>
-      <c r="J9" s="69"/>
-      <c r="K9" s="69"/>
+      <c r="J9" s="86"/>
+      <c r="K9" s="86"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="64" t="s">
+      <c r="A11" s="89" t="s">
         <v>75</v>
       </c>
-      <c r="B11" s="64" t="s">
+      <c r="B11" s="89" t="s">
         <v>76</v>
       </c>
-      <c r="C11" s="64" t="s">
+      <c r="C11" s="89" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="65" t="s">
+      <c r="D11" s="90" t="s">
         <v>77</v>
       </c>
-      <c r="E11" s="65"/>
-      <c r="F11" s="65"/>
-      <c r="G11" s="65" t="s">
+      <c r="E11" s="90"/>
+      <c r="F11" s="90"/>
+      <c r="G11" s="90" t="s">
         <v>78</v>
       </c>
-      <c r="H11" s="65"/>
-      <c r="I11" s="65"/>
-      <c r="J11" s="64" t="s">
+      <c r="H11" s="90"/>
+      <c r="I11" s="90"/>
+      <c r="J11" s="89" t="s">
         <v>79</v>
       </c>
-      <c r="K11" s="63" t="s">
+      <c r="K11" s="88" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="64"/>
-      <c r="B12" s="64"/>
-      <c r="C12" s="64"/>
+      <c r="A12" s="89"/>
+      <c r="B12" s="89"/>
+      <c r="C12" s="89"/>
       <c r="D12" s="47" t="s">
         <v>81</v>
       </c>
@@ -3807,8 +3807,8 @@
       <c r="I12" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="J12" s="64"/>
-      <c r="K12" s="63"/>
+      <c r="J12" s="89"/>
+      <c r="K12" s="88"/>
     </row>
     <row r="13" spans="1:13" s="43" customFormat="1" ht="126.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="48">
@@ -5020,6 +5020,19 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="I9:K9"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="A1:K1"/>
@@ -5027,19 +5040,6 @@
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A5:K5"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:J12"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5072,113 +5072,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="74" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
+      <c r="F1" s="74"/>
+      <c r="G1" s="74"/>
+      <c r="H1" s="74"/>
+      <c r="I1" s="74"/>
+      <c r="J1" s="74"/>
+      <c r="K1" s="74"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="79" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
-      <c r="J2" s="79"/>
-      <c r="K2" s="79"/>
+      <c r="A2" s="75" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="75"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="75"/>
+      <c r="F2" s="75"/>
+      <c r="G2" s="75"/>
+      <c r="H2" s="75"/>
+      <c r="I2" s="75"/>
+      <c r="J2" s="75"/>
+      <c r="K2" s="75"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="80" t="s">
+      <c r="A3" s="76" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="80"/>
-      <c r="C3" s="80"/>
-      <c r="D3" s="80"/>
-      <c r="E3" s="80"/>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
-      <c r="H3" s="80"/>
-      <c r="I3" s="80"/>
-      <c r="J3" s="80"/>
-      <c r="K3" s="80"/>
+      <c r="B3" s="76"/>
+      <c r="C3" s="76"/>
+      <c r="D3" s="76"/>
+      <c r="E3" s="76"/>
+      <c r="F3" s="76"/>
+      <c r="G3" s="76"/>
+      <c r="H3" s="76"/>
+      <c r="I3" s="76"/>
+      <c r="J3" s="76"/>
+      <c r="K3" s="76"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="80" t="s">
+      <c r="A4" s="76" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="80"/>
-      <c r="C4" s="80"/>
-      <c r="D4" s="80"/>
-      <c r="E4" s="80"/>
-      <c r="F4" s="80"/>
-      <c r="G4" s="80"/>
-      <c r="H4" s="80"/>
-      <c r="I4" s="80"/>
-      <c r="J4" s="80"/>
-      <c r="K4" s="80"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="76"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="76"/>
+      <c r="F4" s="76"/>
+      <c r="G4" s="76"/>
+      <c r="H4" s="76"/>
+      <c r="I4" s="76"/>
+      <c r="J4" s="76"/>
+      <c r="K4" s="76"/>
     </row>
     <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="81" t="s">
+      <c r="A5" s="77" t="s">
         <v>85</v>
       </c>
-      <c r="B5" s="81"/>
-      <c r="C5" s="81"/>
-      <c r="D5" s="81"/>
-      <c r="E5" s="81"/>
-      <c r="F5" s="81"/>
-      <c r="G5" s="81"/>
-      <c r="H5" s="81"/>
-      <c r="I5" s="81"/>
-      <c r="J5" s="81"/>
-      <c r="K5" s="81"/>
+      <c r="B5" s="77"/>
+      <c r="C5" s="77"/>
+      <c r="D5" s="77"/>
+      <c r="E5" s="77"/>
+      <c r="F5" s="77"/>
+      <c r="G5" s="77"/>
+      <c r="H5" s="77"/>
+      <c r="I5" s="77"/>
+      <c r="J5" s="77"/>
+      <c r="K5" s="77"/>
     </row>
     <row r="6" spans="1:11" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="68" t="s">
+      <c r="A6" s="72" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="68"/>
-      <c r="C6" s="68"/>
-      <c r="D6" s="68"/>
-      <c r="E6" s="68"/>
-      <c r="F6" s="68"/>
+      <c r="B6" s="72"/>
+      <c r="C6" s="72"/>
+      <c r="D6" s="72"/>
+      <c r="E6" s="72"/>
+      <c r="F6" s="72"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="77" t="s">
+      <c r="H6" s="73" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="77"/>
-      <c r="J6" s="77"/>
-      <c r="K6" s="77"/>
+      <c r="I6" s="73"/>
+      <c r="J6" s="73"/>
+      <c r="K6" s="73"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="84" t="s">
+      <c r="A7" s="67" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="84"/>
-      <c r="C7" s="84"/>
-      <c r="D7" s="84"/>
-      <c r="E7" s="84"/>
-      <c r="F7" s="84"/>
+      <c r="B7" s="67"/>
+      <c r="C7" s="67"/>
+      <c r="D7" s="67"/>
+      <c r="E7" s="67"/>
+      <c r="F7" s="67"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="85" t="s">
+      <c r="H7" s="68" t="s">
         <v>88</v>
       </c>
-      <c r="I7" s="85"/>
-      <c r="J7" s="85"/>
-      <c r="K7" s="85"/>
+      <c r="I7" s="68"/>
+      <c r="J7" s="68"/>
+      <c r="K7" s="68"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
@@ -5571,7 +5571,7 @@
       <c r="J22" s="17"/>
       <c r="K22" s="17"/>
     </row>
-    <row r="23" spans="1:13" ht="173.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" ht="157.5" x14ac:dyDescent="0.25">
       <c r="A23" s="16">
         <v>2</v>
       </c>
@@ -5676,7 +5676,7 @@
       <c r="J27" s="17"/>
       <c r="K27" s="17"/>
     </row>
-    <row r="28" spans="1:13" ht="110.25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" ht="94.5" x14ac:dyDescent="0.25">
       <c r="A28" s="16">
         <v>3</v>
       </c>
@@ -6052,7 +6052,7 @@
       <c r="J42" s="17"/>
       <c r="K42" s="17"/>
     </row>
-    <row r="43" spans="1:11" ht="94.5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A43" s="16">
         <v>4</v>
       </c>
@@ -7458,7 +7458,7 @@
       <c r="J104" s="17"/>
       <c r="K104" s="17"/>
     </row>
-    <row r="105" spans="1:14" ht="150" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:14" ht="135" x14ac:dyDescent="0.25">
       <c r="A105" s="16">
         <v>8</v>
       </c>
@@ -7805,11 +7805,11 @@
       <c r="B122" s="27" t="s">
         <v>84</v>
       </c>
-      <c r="C122" s="82">
+      <c r="C122" s="65">
         <f>J120</f>
         <v>569089.07039927552</v>
       </c>
-      <c r="D122" s="83"/>
+      <c r="D122" s="66"/>
       <c r="E122" s="9">
         <v>100</v>
       </c>
@@ -7825,21 +7825,21 @@
       <c r="B123" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C123" s="86">
+      <c r="C123" s="69">
         <v>500000</v>
       </c>
-      <c r="D123" s="87"/>
+      <c r="D123" s="70"/>
       <c r="E123" s="9"/>
     </row>
     <row r="124" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B124" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C124" s="86">
+      <c r="C124" s="69">
         <f>C123-C126-C127</f>
         <v>475000</v>
       </c>
-      <c r="D124" s="87"/>
+      <c r="D124" s="70"/>
       <c r="E124" s="9">
         <f>C124/C122*100</f>
         <v>83.466723349077469</v>
@@ -7849,11 +7849,11 @@
       <c r="B125" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="C125" s="88">
+      <c r="C125" s="71">
         <f>C122-C124</f>
         <v>94089.070399275515</v>
       </c>
-      <c r="D125" s="88"/>
+      <c r="D125" s="71"/>
       <c r="E125" s="9">
         <f>100-E124</f>
         <v>16.533276650922531</v>
@@ -7863,11 +7863,11 @@
       <c r="B126" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C126" s="82">
+      <c r="C126" s="65">
         <f>C123*0.03</f>
         <v>15000</v>
       </c>
-      <c r="D126" s="83"/>
+      <c r="D126" s="66"/>
       <c r="E126" s="9">
         <v>3</v>
       </c>
@@ -7876,17 +7876,24 @@
       <c r="B127" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C127" s="82">
+      <c r="C127" s="65">
         <f>C123*0.02</f>
         <v>10000</v>
       </c>
-      <c r="D127" s="83"/>
+      <c r="D127" s="66"/>
       <c r="E127" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C126:D126"/>
     <mergeCell ref="C127:D127"/>
     <mergeCell ref="A7:F7"/>
@@ -7895,13 +7902,6 @@
     <mergeCell ref="C123:D123"/>
     <mergeCell ref="C124:D124"/>
     <mergeCell ref="C125:D125"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
@@ -7930,108 +7930,108 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="74" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
+      <c r="F1" s="74"/>
+      <c r="G1" s="74"/>
+      <c r="H1" s="74"/>
+      <c r="I1" s="74"/>
+      <c r="J1" s="74"/>
+      <c r="K1" s="74"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="79" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
-      <c r="J2" s="79"/>
-      <c r="K2" s="79"/>
+      <c r="A2" s="75" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="75"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="75"/>
+      <c r="F2" s="75"/>
+      <c r="G2" s="75"/>
+      <c r="H2" s="75"/>
+      <c r="I2" s="75"/>
+      <c r="J2" s="75"/>
+      <c r="K2" s="75"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="80" t="s">
+      <c r="A3" s="76" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="80"/>
-      <c r="C3" s="80"/>
-      <c r="D3" s="80"/>
-      <c r="E3" s="80"/>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
-      <c r="H3" s="80"/>
-      <c r="I3" s="80"/>
-      <c r="J3" s="80"/>
-      <c r="K3" s="80"/>
+      <c r="B3" s="76"/>
+      <c r="C3" s="76"/>
+      <c r="D3" s="76"/>
+      <c r="E3" s="76"/>
+      <c r="F3" s="76"/>
+      <c r="G3" s="76"/>
+      <c r="H3" s="76"/>
+      <c r="I3" s="76"/>
+      <c r="J3" s="76"/>
+      <c r="K3" s="76"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="80" t="s">
+      <c r="A4" s="76" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="80"/>
-      <c r="C4" s="80"/>
-      <c r="D4" s="80"/>
-      <c r="E4" s="80"/>
-      <c r="F4" s="80"/>
-      <c r="G4" s="80"/>
-      <c r="H4" s="80"/>
-      <c r="I4" s="80"/>
-      <c r="J4" s="80"/>
-      <c r="K4" s="80"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="76"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="76"/>
+      <c r="F4" s="76"/>
+      <c r="G4" s="76"/>
+      <c r="H4" s="76"/>
+      <c r="I4" s="76"/>
+      <c r="J4" s="76"/>
+      <c r="K4" s="76"/>
     </row>
     <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="81" t="s">
+      <c r="A5" s="77" t="s">
         <v>86</v>
       </c>
-      <c r="B5" s="81"/>
-      <c r="C5" s="81"/>
-      <c r="D5" s="81"/>
-      <c r="E5" s="81"/>
-      <c r="F5" s="81"/>
-      <c r="G5" s="81"/>
-      <c r="H5" s="81"/>
-      <c r="I5" s="81"/>
-      <c r="J5" s="81"/>
-      <c r="K5" s="81"/>
+      <c r="B5" s="77"/>
+      <c r="C5" s="77"/>
+      <c r="D5" s="77"/>
+      <c r="E5" s="77"/>
+      <c r="F5" s="77"/>
+      <c r="G5" s="77"/>
+      <c r="H5" s="77"/>
+      <c r="I5" s="77"/>
+      <c r="J5" s="77"/>
+      <c r="K5" s="77"/>
     </row>
     <row r="6" spans="1:11" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="68" t="s">
+      <c r="A6" s="72" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="68"/>
-      <c r="C6" s="68"/>
-      <c r="D6" s="68"/>
-      <c r="E6" s="68"/>
-      <c r="F6" s="68"/>
+      <c r="B6" s="72"/>
+      <c r="C6" s="72"/>
+      <c r="D6" s="72"/>
+      <c r="E6" s="72"/>
+      <c r="F6" s="72"/>
       <c r="G6" s="10"/>
-      <c r="I6" s="90"/>
-      <c r="J6" s="90"/>
+      <c r="I6" s="64"/>
+      <c r="J6" s="64"/>
       <c r="K6" s="42" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="84" t="s">
+      <c r="A7" s="67" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="84"/>
-      <c r="C7" s="84"/>
-      <c r="D7" s="84"/>
-      <c r="E7" s="84"/>
-      <c r="F7" s="84"/>
+      <c r="B7" s="67"/>
+      <c r="C7" s="67"/>
+      <c r="D7" s="67"/>
+      <c r="E7" s="67"/>
+      <c r="F7" s="67"/>
       <c r="G7" s="11"/>
-      <c r="I7" s="89"/>
-      <c r="J7" s="89"/>
+      <c r="I7" s="63"/>
+      <c r="J7" s="63"/>
       <c r="K7" s="41" t="s">
         <v>88</v>
       </c>
@@ -10314,7 +10314,7 @@
       <c r="J104" s="17"/>
       <c r="K104" s="17"/>
     </row>
-    <row r="105" spans="1:14" ht="120" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:14" ht="105" x14ac:dyDescent="0.25">
       <c r="A105" s="16">
         <v>8</v>
       </c>
@@ -10661,11 +10661,11 @@
       <c r="B122" s="27" t="s">
         <v>84</v>
       </c>
-      <c r="C122" s="82">
+      <c r="C122" s="65">
         <f>J120</f>
         <v>569089.07039927552</v>
       </c>
-      <c r="D122" s="83"/>
+      <c r="D122" s="66"/>
       <c r="E122" s="9">
         <v>100</v>
       </c>
@@ -10681,21 +10681,21 @@
       <c r="B123" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C123" s="86">
+      <c r="C123" s="69">
         <v>500000</v>
       </c>
-      <c r="D123" s="87"/>
+      <c r="D123" s="70"/>
       <c r="E123" s="9"/>
     </row>
     <row r="124" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="B124" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C124" s="86">
+      <c r="C124" s="69">
         <f>C123-C126-C127</f>
         <v>475000</v>
       </c>
-      <c r="D124" s="87"/>
+      <c r="D124" s="70"/>
       <c r="E124" s="9">
         <f>C124/C122*100</f>
         <v>83.466723349077469</v>
@@ -10705,11 +10705,11 @@
       <c r="B125" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="C125" s="88">
+      <c r="C125" s="71">
         <f>C122-C124</f>
         <v>94089.070399275515</v>
       </c>
-      <c r="D125" s="88"/>
+      <c r="D125" s="71"/>
       <c r="E125" s="9">
         <f>100-E124</f>
         <v>16.533276650922531</v>
@@ -10719,11 +10719,11 @@
       <c r="B126" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C126" s="82">
+      <c r="C126" s="65">
         <f>C123*0.03</f>
         <v>15000</v>
       </c>
-      <c r="D126" s="83"/>
+      <c r="D126" s="66"/>
       <c r="E126" s="9">
         <v>3</v>
       </c>
@@ -10732,17 +10732,23 @@
       <c r="B127" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C127" s="82">
+      <c r="C127" s="65">
         <f>C123*0.02</f>
         <v>10000</v>
       </c>
-      <c r="D127" s="83"/>
+      <c r="D127" s="66"/>
       <c r="E127" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C126:D126"/>
     <mergeCell ref="C127:D127"/>
     <mergeCell ref="A7:F7"/>
@@ -10750,12 +10756,6 @@
     <mergeCell ref="C123:D123"/>
     <mergeCell ref="C124:D124"/>
     <mergeCell ref="C125:D125"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A6:F6"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="90" orientation="portrait" verticalDpi="1200" r:id="rId1"/>

</xml_diff>